<commit_message>
Unstratefied MS Registry data 24 Oct
</commit_message>
<xml_diff>
--- a/data-raw/ExponentialSurvivalModels 21Oct2024.xlsx
+++ b/data-raw/ExponentialSurvivalModels 21Oct2024.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://uob.sharepoint.com/teams/grp-Bristol_TAG-MTA-MS/Shared Documents/MTA-MS/Working Folder_HE/MS Models/Git Repo/MS-MTA/data-raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{55280907-FD0B-49FF-83BF-FA12A7D5D18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D3CF5A54-F9FF-4F77-9FFE-C3749AEB863E}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{55280907-FD0B-49FF-83BF-FA12A7D5D18F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BAEE230D-2C50-4013-B3C0-452FDDECDAFA}"/>
   <bookViews>
-    <workbookView xWindow="28785" yWindow="-16425" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28785" yWindow="-16425" windowWidth="29040" windowHeight="15720" tabRatio="472" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Models" sheetId="1" r:id="rId1"/>
-    <sheet name="Table 2" sheetId="2" r:id="rId2"/>
+    <sheet name="Models without DMTs" sheetId="3" r:id="rId2"/>
+    <sheet name="Table 2" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -95,7 +96,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="536" uniqueCount="46">
   <si>
     <t>Time to EDSS Increase (RRMS Highly Active)</t>
   </si>
@@ -239,7 +240,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -254,14 +255,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
-    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -277,6 +272,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="3" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.79998168889431442"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -297,8 +298,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -668,7 +669,7 @@
       <c r="B6" s="2">
         <v>0.93328576763113402</v>
       </c>
-      <c r="C6" s="3">
+      <c r="C6">
         <v>-7.2165558831459697E-2</v>
       </c>
       <c r="D6">
@@ -699,7 +700,7 @@
       <c r="B7" s="2">
         <v>0.17821799667817501</v>
       </c>
-      <c r="C7" s="3">
+      <c r="C7">
         <v>3.10170417624735E-2</v>
       </c>
       <c r="D7">
@@ -950,11 +951,11 @@
       </c>
       <c r="M17" s="2"/>
       <c r="N17" s="2" t="str">
-        <f>B17</f>
+        <f t="shared" ref="N17:O19" si="0">B17</f>
         <v>(Intercept)</v>
       </c>
       <c r="O17" s="2" t="str">
-        <f>C17</f>
+        <f t="shared" si="0"/>
         <v>BaselineWebEDSS</v>
       </c>
       <c r="P17" s="2" t="str">
@@ -1001,11 +1002,11 @@
         <v>(Intercept)</v>
       </c>
       <c r="N18" s="2">
-        <f>B18</f>
+        <f t="shared" si="0"/>
         <v>0.263163661794172</v>
       </c>
       <c r="O18" s="2">
-        <f>C18</f>
+        <f t="shared" si="0"/>
         <v>-1.88754009677474E-2</v>
       </c>
       <c r="P18" s="2">
@@ -1052,11 +1053,11 @@
         <v>BaselineWebEDSS</v>
       </c>
       <c r="N19" s="2">
-        <f>B19</f>
+        <f t="shared" si="0"/>
         <v>-1.88754009677474E-2</v>
       </c>
       <c r="O19" s="2">
-        <f>C19</f>
+        <f t="shared" si="0"/>
         <v>5.6405970074095502E-3</v>
       </c>
       <c r="P19" s="2">
@@ -1686,11 +1687,11 @@
       </c>
       <c r="M45" s="2"/>
       <c r="N45" s="2" t="str">
-        <f>B45</f>
+        <f t="shared" ref="N45:O47" si="1">B45</f>
         <v>(Intercept)</v>
       </c>
       <c r="O45" s="2" t="str">
-        <f>C45</f>
+        <f t="shared" si="1"/>
         <v>BaselineWebEDSS</v>
       </c>
       <c r="P45" s="2" t="str">
@@ -1737,11 +1738,11 @@
         <v>(Intercept)</v>
       </c>
       <c r="N46" s="2">
-        <f>B46</f>
+        <f t="shared" si="1"/>
         <v>3.7916845646299997E-2</v>
       </c>
       <c r="O46" s="2">
-        <f>C46</f>
+        <f t="shared" si="1"/>
         <v>-4.2253696820032903E-3</v>
       </c>
       <c r="P46" s="2">
@@ -1788,11 +1789,11 @@
         <v>BaselineWebEDSS</v>
       </c>
       <c r="N47" s="2">
-        <f>B47</f>
+        <f t="shared" si="1"/>
         <v>-4.2253696820032903E-3</v>
       </c>
       <c r="O47" s="2">
-        <f>C47</f>
+        <f t="shared" si="1"/>
         <v>1.53897616595774E-3</v>
       </c>
       <c r="P47" s="2">
@@ -2422,11 +2423,11 @@
       </c>
       <c r="M73" s="2"/>
       <c r="N73" s="2" t="str">
-        <f>B73</f>
+        <f t="shared" ref="N73:O75" si="2">B73</f>
         <v>(Intercept)</v>
       </c>
       <c r="O73" s="2" t="str">
-        <f>C73</f>
+        <f t="shared" si="2"/>
         <v>BaselineWebEDSS</v>
       </c>
       <c r="P73" s="2" t="str">
@@ -2473,11 +2474,11 @@
         <v>(Intercept)</v>
       </c>
       <c r="N74" s="2">
-        <f>B74</f>
+        <f t="shared" si="2"/>
         <v>9.1137145835865199E-2</v>
       </c>
       <c r="O74" s="2">
-        <f>C74</f>
+        <f t="shared" si="2"/>
         <v>-1.04160472332989E-2</v>
       </c>
       <c r="P74" s="2">
@@ -2524,11 +2525,11 @@
         <v>BaselineWebEDSS</v>
       </c>
       <c r="N75" s="2">
-        <f>B75</f>
+        <f t="shared" si="2"/>
         <v>-1.04160472332989E-2</v>
       </c>
       <c r="O75" s="2">
-        <f>C75</f>
+        <f t="shared" si="2"/>
         <v>2.6373740268514898E-3</v>
       </c>
       <c r="P75" s="2">
@@ -3095,7 +3096,7 @@
       <c r="F98">
         <v>0</v>
       </c>
-      <c r="G98" s="4" t="e">
+      <c r="G98" s="3" t="e">
         <v>#NUM!</v>
       </c>
     </row>
@@ -3132,11 +3133,11 @@
       </c>
       <c r="M101" s="2"/>
       <c r="N101" s="2" t="str">
-        <f>B101</f>
+        <f t="shared" ref="N101:O103" si="3">B101</f>
         <v>(Intercept)</v>
       </c>
       <c r="O101" s="2" t="str">
-        <f>C101</f>
+        <f t="shared" si="3"/>
         <v>BaselineWebEDSS</v>
       </c>
       <c r="P101" s="2" t="str">
@@ -3180,11 +3181,11 @@
         <v>(Intercept)</v>
       </c>
       <c r="N102" s="2">
-        <f>B102</f>
+        <f t="shared" si="3"/>
         <v>0.54065168373127903</v>
       </c>
       <c r="O102" s="2">
-        <f>C102</f>
+        <f t="shared" si="3"/>
         <v>-7.1644001823843298E-2</v>
       </c>
       <c r="P102" s="2">
@@ -3228,11 +3229,11 @@
         <v>BaselineWebEDSS</v>
       </c>
       <c r="N103" s="2">
-        <f>B103</f>
+        <f t="shared" si="3"/>
         <v>-7.1644001823843298E-2</v>
       </c>
       <c r="O103" s="2">
-        <f>C103</f>
+        <f t="shared" si="3"/>
         <v>1.23489527367181E-2</v>
       </c>
       <c r="P103" s="2">
@@ -3597,7 +3598,7 @@
       <c r="F120">
         <v>0</v>
       </c>
-      <c r="G120" s="4" t="e">
+      <c r="G120" s="3" t="e">
         <v>#NUM!</v>
       </c>
       <c r="M120" s="2" t="str">
@@ -3628,7 +3629,7 @@
       <c r="F121">
         <v>0</v>
       </c>
-      <c r="G121" s="4" t="e">
+      <c r="G121" s="3" t="e">
         <v>#NUM!</v>
       </c>
     </row>
@@ -3651,7 +3652,7 @@
       <c r="F122">
         <v>0</v>
       </c>
-      <c r="G122" s="4" t="e">
+      <c r="G122" s="3" t="e">
         <v>#NUM!</v>
       </c>
     </row>
@@ -3743,7 +3744,7 @@
       <c r="F126">
         <v>0</v>
       </c>
-      <c r="G126" s="4" t="e">
+      <c r="G126" s="3" t="e">
         <v>#NUM!</v>
       </c>
     </row>
@@ -3780,11 +3781,11 @@
       </c>
       <c r="M129" s="2"/>
       <c r="N129" s="2" t="str">
-        <f>B129</f>
+        <f t="shared" ref="N129:O131" si="4">B129</f>
         <v>(Intercept)</v>
       </c>
       <c r="O129" s="2" t="str">
-        <f>C129</f>
+        <f t="shared" si="4"/>
         <v>BaselineWebEDSS</v>
       </c>
       <c r="P129" s="2" t="str">
@@ -3828,11 +3829,11 @@
         <v>(Intercept)</v>
       </c>
       <c r="N130" s="2">
-        <f>B130</f>
+        <f t="shared" si="4"/>
         <v>8.4002318710323802</v>
       </c>
       <c r="O130" s="2">
-        <f>C130</f>
+        <f t="shared" si="4"/>
         <v>-1.2179985752128999</v>
       </c>
       <c r="P130" s="2">
@@ -3876,11 +3877,11 @@
         <v>BaselineWebEDSS</v>
       </c>
       <c r="N131" s="2">
-        <f>B131</f>
+        <f t="shared" si="4"/>
         <v>-1.2179985752128999</v>
       </c>
       <c r="O131" s="2">
-        <f>C131</f>
+        <f t="shared" si="4"/>
         <v>0.180179605359056</v>
       </c>
       <c r="P131" s="2">
@@ -4245,7 +4246,7 @@
       <c r="F148">
         <v>0</v>
       </c>
-      <c r="G148" s="4" t="e">
+      <c r="G148" s="3" t="e">
         <v>#NUM!</v>
       </c>
       <c r="M148" s="2" t="str">
@@ -4402,11 +4403,11 @@
       </c>
       <c r="M157" s="2"/>
       <c r="N157" s="2" t="str">
-        <f>B157</f>
+        <f t="shared" ref="N157:O159" si="5">B157</f>
         <v>(Intercept)</v>
       </c>
       <c r="O157" s="2" t="str">
-        <f>C157</f>
+        <f t="shared" si="5"/>
         <v>BaselineWebEDSS</v>
       </c>
       <c r="P157" s="2" t="str">
@@ -4447,11 +4448,11 @@
         <v>(Intercept)</v>
       </c>
       <c r="N158" s="2">
-        <f>B158</f>
+        <f t="shared" si="5"/>
         <v>0.93094557897014996</v>
       </c>
       <c r="O158" s="2">
-        <f>C158</f>
+        <f t="shared" si="5"/>
         <v>-0.140770879719954</v>
       </c>
       <c r="P158" s="2">
@@ -4492,11 +4493,11 @@
         <v>BaselineWebEDSS</v>
       </c>
       <c r="N159" s="2">
-        <f>B159</f>
+        <f t="shared" si="5"/>
         <v>-0.140770879719954</v>
       </c>
       <c r="O159" s="2">
-        <f>C159</f>
+        <f t="shared" si="5"/>
         <v>2.2494511636344E-2</v>
       </c>
       <c r="P159" s="2">
@@ -5020,11 +5021,11 @@
       </c>
       <c r="M185" s="2"/>
       <c r="N185" s="2" t="str">
-        <f>B185</f>
+        <f t="shared" ref="N185:O187" si="6">B185</f>
         <v>(Intercept)</v>
       </c>
       <c r="O185" s="2" t="str">
-        <f>C185</f>
+        <f t="shared" si="6"/>
         <v>BaselineWebEDSS</v>
       </c>
       <c r="P185" s="2" t="str">
@@ -5071,11 +5072,11 @@
         <v>(Intercept)</v>
       </c>
       <c r="N186" s="2">
-        <f>B186</f>
+        <f t="shared" si="6"/>
         <v>0.17602810350735501</v>
       </c>
       <c r="O186" s="2">
-        <f>C186</f>
+        <f t="shared" si="6"/>
         <v>-2.1262047871894101E-2</v>
       </c>
       <c r="P186" s="2">
@@ -5122,11 +5123,11 @@
         <v>BaselineWebEDSS</v>
       </c>
       <c r="N187" s="2">
-        <f>B187</f>
+        <f t="shared" si="6"/>
         <v>-2.1262047871894101E-2</v>
       </c>
       <c r="O187" s="2">
-        <f>C187</f>
+        <f t="shared" si="6"/>
         <v>8.8593274810134792E-3</v>
       </c>
       <c r="P187" s="2">
@@ -5756,11 +5757,11 @@
       </c>
       <c r="M213" s="2"/>
       <c r="N213" s="2" t="str">
-        <f>B213</f>
+        <f t="shared" ref="N213:O215" si="7">B213</f>
         <v>(Intercept)</v>
       </c>
       <c r="O213" s="2" t="str">
-        <f>C213</f>
+        <f t="shared" si="7"/>
         <v>BaselineWebEDSS</v>
       </c>
       <c r="P213" s="2" t="str">
@@ -5807,11 +5808,11 @@
         <v>(Intercept)</v>
       </c>
       <c r="N214" s="2">
-        <f>B214</f>
+        <f t="shared" si="7"/>
         <v>5.3104247945483497E-2</v>
       </c>
       <c r="O214" s="2">
-        <f>C214</f>
+        <f t="shared" si="7"/>
         <v>-7.4094810243937803E-3</v>
       </c>
       <c r="P214" s="2">
@@ -5858,11 +5859,11 @@
         <v>BaselineWebEDSS</v>
       </c>
       <c r="N215" s="2">
-        <f>B215</f>
+        <f t="shared" si="7"/>
         <v>-7.4094810243937803E-3</v>
       </c>
       <c r="O215" s="2">
-        <f>C215</f>
+        <f t="shared" si="7"/>
         <v>1.9119732942815401E-3</v>
       </c>
       <c r="P215" s="2">
@@ -6414,11 +6415,11 @@
       </c>
       <c r="M241" s="2"/>
       <c r="N241" s="2" t="str">
-        <f>B241</f>
+        <f t="shared" ref="N241:O243" si="8">B241</f>
         <v>(Intercept)</v>
       </c>
       <c r="O241" s="2" t="str">
-        <f>C241</f>
+        <f t="shared" si="8"/>
         <v>BaselineWebEDSS</v>
       </c>
       <c r="P241" s="2" t="str">
@@ -6456,11 +6457,11 @@
         <v>(Intercept)</v>
       </c>
       <c r="N242" s="2">
-        <f>B242</f>
+        <f t="shared" si="8"/>
         <v>0.519597791750535</v>
       </c>
       <c r="O242" s="2">
-        <f>C242</f>
+        <f t="shared" si="8"/>
         <v>-8.1783357619617997E-2</v>
       </c>
       <c r="P242" s="2">
@@ -6498,11 +6499,11 @@
         <v>BaselineWebEDSS</v>
       </c>
       <c r="N243" s="2">
-        <f>B243</f>
+        <f t="shared" si="8"/>
         <v>-8.1783357619617997E-2</v>
       </c>
       <c r="O243" s="2">
-        <f>C243</f>
+        <f t="shared" si="8"/>
         <v>1.4106533490992E-2</v>
       </c>
       <c r="P243" s="2">
@@ -6932,11 +6933,11 @@
       </c>
       <c r="M269" s="2"/>
       <c r="N269" s="2" t="str">
-        <f>B269</f>
+        <f t="shared" ref="N269:O271" si="9">B269</f>
         <v>(Intercept)</v>
       </c>
       <c r="O269" s="2" t="str">
-        <f>C269</f>
+        <f t="shared" si="9"/>
         <v>BaselineWebEDSS</v>
       </c>
       <c r="P269" s="2" t="str">
@@ -6977,11 +6978,11 @@
         <v>(Intercept)</v>
       </c>
       <c r="N270" s="2">
-        <f>B270</f>
+        <f t="shared" si="9"/>
         <v>0.14377939322371899</v>
       </c>
       <c r="O270" s="2">
-        <f>C270</f>
+        <f t="shared" si="9"/>
         <v>-2.1761720330557101E-2</v>
       </c>
       <c r="P270" s="2">
@@ -7022,11 +7023,11 @@
         <v>BaselineWebEDSS</v>
       </c>
       <c r="N271" s="2">
-        <f>B271</f>
+        <f t="shared" si="9"/>
         <v>-2.1761720330557101E-2</v>
       </c>
       <c r="O271" s="2">
-        <f>C271</f>
+        <f t="shared" si="9"/>
         <v>3.5399508123902502E-3</v>
       </c>
       <c r="P271" s="2">
@@ -7232,11 +7233,962 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{25C87838-3AF5-446C-9D66-DFC9725BB240}">
+  <dimension ref="A1:G103"/>
+  <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B1" s="4"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" t="s">
+        <v>4</v>
+      </c>
+      <c r="D5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E5" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B6" s="4">
+        <v>3.5071491149592999</v>
+      </c>
+      <c r="C6">
+        <v>3.0753462564886398</v>
+      </c>
+      <c r="D6">
+        <v>3.9389519734299498</v>
+      </c>
+      <c r="E6">
+        <v>33.353046414763597</v>
+      </c>
+      <c r="F6">
+        <v>21.6573796215927</v>
+      </c>
+      <c r="G6">
+        <v>51.364741468366397</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" s="4">
+        <v>-0.137924847521192</v>
+      </c>
+      <c r="C7">
+        <v>-0.23444851876497499</v>
+      </c>
+      <c r="D7">
+        <v>-4.1401176277408899E-2</v>
+      </c>
+      <c r="E7">
+        <v>0.87116415943176795</v>
+      </c>
+      <c r="F7">
+        <v>0.79100695485813599</v>
+      </c>
+      <c r="G7">
+        <v>0.95944414649877496</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B11" s="4">
+        <v>4.85372139300288E-2</v>
+      </c>
+      <c r="C11" s="4">
+        <v>-9.9457478203662103E-3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" s="4">
+        <v>-9.9457478203662103E-3</v>
+      </c>
+      <c r="C12" s="4">
+        <v>2.4253335894654799E-3</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="B14" s="4"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B18" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" t="s">
+        <v>4</v>
+      </c>
+      <c r="D18" t="s">
+        <v>5</v>
+      </c>
+      <c r="E18" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" t="s">
+        <v>7</v>
+      </c>
+      <c r="G18" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B19" s="4">
+        <v>1.88774266700013</v>
+      </c>
+      <c r="C19">
+        <v>0.62774208146017296</v>
+      </c>
+      <c r="D19">
+        <v>3.1477432525400801</v>
+      </c>
+      <c r="E19">
+        <v>6.6044434136680303</v>
+      </c>
+      <c r="F19">
+        <v>1.87337587014008</v>
+      </c>
+      <c r="G19">
+        <v>23.283460356026399</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B20" s="4">
+        <v>0.20440888444584299</v>
+      </c>
+      <c r="C20">
+        <v>-1.2122078735466E-2</v>
+      </c>
+      <c r="D20">
+        <v>0.42093984762715098</v>
+      </c>
+      <c r="E20">
+        <v>1.22679967022134</v>
+      </c>
+      <c r="F20">
+        <v>0.98795109767909906</v>
+      </c>
+      <c r="G20">
+        <v>1.52339263997057</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B24" s="4">
+        <v>0.41328087834979299</v>
+      </c>
+      <c r="C24" s="4">
+        <v>-6.8523311664260303E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B25" s="4">
+        <v>-6.8523311664260303E-2</v>
+      </c>
+      <c r="C25" s="4">
+        <v>1.22051700160496E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" s="4"/>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B31" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C31" t="s">
+        <v>4</v>
+      </c>
+      <c r="D31" t="s">
+        <v>5</v>
+      </c>
+      <c r="E31" t="s">
+        <v>6</v>
+      </c>
+      <c r="F31" t="s">
+        <v>7</v>
+      </c>
+      <c r="G31" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B32" s="4">
+        <v>10.3405958779194</v>
+      </c>
+      <c r="C32">
+        <v>5.0615857862878801</v>
+      </c>
+      <c r="D32">
+        <v>15.6196059695509</v>
+      </c>
+      <c r="E32">
+        <v>30964.4755981462</v>
+      </c>
+      <c r="F32">
+        <v>157.84061945590099</v>
+      </c>
+      <c r="G32">
+        <v>6074474.0636048401</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B33" s="4">
+        <v>-0.99003801329779295</v>
+      </c>
+      <c r="C33">
+        <v>-1.78080573929592</v>
+      </c>
+      <c r="D33">
+        <v>-0.199270287299667</v>
+      </c>
+      <c r="E33">
+        <v>0.37156256643509999</v>
+      </c>
+      <c r="F33">
+        <v>0.168502323613127</v>
+      </c>
+      <c r="G33">
+        <v>0.81932840933881801</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B36" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C36" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" s="4">
+        <v>7.2545220053958497</v>
+      </c>
+      <c r="C37" s="4">
+        <v>-1.0813258932986201</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B38" s="4">
+        <v>-1.0813258932986201</v>
+      </c>
+      <c r="C38" s="4">
+        <v>0.162780242003806</v>
+      </c>
+    </row>
+    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A40" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B40" s="4"/>
+    </row>
+    <row r="42" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A44" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B44" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C44" t="s">
+        <v>4</v>
+      </c>
+      <c r="D44" t="s">
+        <v>5</v>
+      </c>
+      <c r="E44" t="s">
+        <v>6</v>
+      </c>
+      <c r="F44" t="s">
+        <v>7</v>
+      </c>
+      <c r="G44" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A45" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B45" s="4">
+        <v>4.8340183103396397</v>
+      </c>
+      <c r="C45">
+        <v>3.0069738018935301</v>
+      </c>
+      <c r="D45">
+        <v>6.6610628187857603</v>
+      </c>
+      <c r="E45">
+        <v>125.71510938726701</v>
+      </c>
+      <c r="F45">
+        <v>20.226099035102902</v>
+      </c>
+      <c r="G45">
+        <v>781.38096233107899</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A46" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B46" s="4">
+        <v>-6.7234350635073298E-2</v>
+      </c>
+      <c r="C46">
+        <v>-0.35717363632258903</v>
+      </c>
+      <c r="D46">
+        <v>0.22270493505244199</v>
+      </c>
+      <c r="E46">
+        <v>0.93497606342598305</v>
+      </c>
+      <c r="F46">
+        <v>0.69965100235976596</v>
+      </c>
+      <c r="G46">
+        <v>1.24945184989535</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A48" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="49" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A49" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B49" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C49" s="4" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="50" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A50" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="B50" s="4">
+        <v>0.86896457612942402</v>
+      </c>
+      <c r="C50" s="4">
+        <v>-0.13573720835203701</v>
+      </c>
+    </row>
+    <row r="51" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A51" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B51" s="4">
+        <v>-0.13573720835203701</v>
+      </c>
+      <c r="C51" s="4">
+        <v>2.1883558644993299E-2</v>
+      </c>
+    </row>
+    <row r="53" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A53" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="57" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>2</v>
+      </c>
+      <c r="B57" t="s">
+        <v>3</v>
+      </c>
+      <c r="C57" t="s">
+        <v>4</v>
+      </c>
+      <c r="D57" t="s">
+        <v>5</v>
+      </c>
+      <c r="E57" t="s">
+        <v>6</v>
+      </c>
+      <c r="F57" t="s">
+        <v>7</v>
+      </c>
+      <c r="G57" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="58" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>9</v>
+      </c>
+      <c r="B58">
+        <v>2.3222247091040198</v>
+      </c>
+      <c r="C58">
+        <v>1.71179033087052</v>
+      </c>
+      <c r="D58">
+        <v>2.93265908733752</v>
+      </c>
+      <c r="E58">
+        <v>10.1983374214138</v>
+      </c>
+      <c r="F58">
+        <v>5.5388690142772798</v>
+      </c>
+      <c r="G58">
+        <v>18.777495169666899</v>
+      </c>
+    </row>
+    <row r="59" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>10</v>
+      </c>
+      <c r="B59">
+        <v>7.1990119044455902E-2</v>
+      </c>
+      <c r="C59">
+        <v>-8.1144310098238304E-2</v>
+      </c>
+      <c r="D59">
+        <v>0.22512454818715</v>
+      </c>
+      <c r="E59">
+        <v>1.0746447254945899</v>
+      </c>
+      <c r="F59">
+        <v>0.92206061918446702</v>
+      </c>
+      <c r="G59">
+        <v>1.25247870042947</v>
+      </c>
+    </row>
+    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>2</v>
+      </c>
+      <c r="B62" t="s">
+        <v>9</v>
+      </c>
+      <c r="C62" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>9</v>
+      </c>
+      <c r="B63">
+        <v>9.7002245116346197E-2</v>
+      </c>
+      <c r="C63">
+        <v>-2.1365720847401501E-2</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>10</v>
+      </c>
+      <c r="B64">
+        <v>-2.1365720847401501E-2</v>
+      </c>
+      <c r="C64">
+        <v>6.10449167449921E-3</v>
+      </c>
+    </row>
+    <row r="66" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>2</v>
+      </c>
+      <c r="B70" t="s">
+        <v>3</v>
+      </c>
+      <c r="C70" t="s">
+        <v>4</v>
+      </c>
+      <c r="D70" t="s">
+        <v>5</v>
+      </c>
+      <c r="E70" t="s">
+        <v>6</v>
+      </c>
+      <c r="F70" t="s">
+        <v>7</v>
+      </c>
+      <c r="G70" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>9</v>
+      </c>
+      <c r="B71">
+        <v>2.5660254758347598</v>
+      </c>
+      <c r="C71">
+        <v>2.1959158728185102</v>
+      </c>
+      <c r="D71">
+        <v>2.9361350788510099</v>
+      </c>
+      <c r="E71">
+        <v>13.0139970687526</v>
+      </c>
+      <c r="F71">
+        <v>8.9882293631634091</v>
+      </c>
+      <c r="G71">
+        <v>18.842879154776298</v>
+      </c>
+    </row>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>10</v>
+      </c>
+      <c r="B72">
+        <v>6.0044925807668202E-2</v>
+      </c>
+      <c r="C72">
+        <v>-2.2439633930619599E-2</v>
+      </c>
+      <c r="D72">
+        <v>0.14252948554595599</v>
+      </c>
+      <c r="E72">
+        <v>1.06188425148141</v>
+      </c>
+      <c r="F72">
+        <v>0.97781026197388698</v>
+      </c>
+      <c r="G72">
+        <v>1.15318708280681</v>
+      </c>
+    </row>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>2</v>
+      </c>
+      <c r="B75" t="s">
+        <v>9</v>
+      </c>
+      <c r="C75" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>9</v>
+      </c>
+      <c r="B76">
+        <v>3.5658619456473202E-2</v>
+      </c>
+      <c r="C76">
+        <v>-7.2311870350503099E-3</v>
+      </c>
+    </row>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>10</v>
+      </c>
+      <c r="B77">
+        <v>-7.2311870350503099E-3</v>
+      </c>
+      <c r="C77">
+        <v>1.77112469840033E-3</v>
+      </c>
+    </row>
+    <row r="79" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A79" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="81" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A81" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A83" t="s">
+        <v>2</v>
+      </c>
+      <c r="B83" t="s">
+        <v>3</v>
+      </c>
+      <c r="C83" t="s">
+        <v>4</v>
+      </c>
+      <c r="D83" t="s">
+        <v>5</v>
+      </c>
+      <c r="E83" t="s">
+        <v>6</v>
+      </c>
+      <c r="F83" t="s">
+        <v>7</v>
+      </c>
+      <c r="G83" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="84" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A84" t="s">
+        <v>9</v>
+      </c>
+      <c r="B84">
+        <v>2.5771996210403101</v>
+      </c>
+      <c r="C84">
+        <v>1.2622706471998599</v>
+      </c>
+      <c r="D84">
+        <v>3.89212859488077</v>
+      </c>
+      <c r="E84">
+        <v>13.1602328701441</v>
+      </c>
+      <c r="F84">
+        <v>3.5334355709289</v>
+      </c>
+      <c r="G84">
+        <v>49.015108870625397</v>
+      </c>
+    </row>
+    <row r="85" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A85" t="s">
+        <v>10</v>
+      </c>
+      <c r="B85">
+        <v>-6.7799597797217103E-3</v>
+      </c>
+      <c r="C85">
+        <v>-0.22522604378681299</v>
+      </c>
+      <c r="D85">
+        <v>0.21166612422736999</v>
+      </c>
+      <c r="E85">
+        <v>0.99324297229214198</v>
+      </c>
+      <c r="F85">
+        <v>0.79833573952833004</v>
+      </c>
+      <c r="G85">
+        <v>1.2357352341392001</v>
+      </c>
+    </row>
+    <row r="87" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A87" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="88" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A88" t="s">
+        <v>2</v>
+      </c>
+      <c r="B88" t="s">
+        <v>9</v>
+      </c>
+      <c r="C88" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="89" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A89" t="s">
+        <v>9</v>
+      </c>
+      <c r="B89">
+        <v>0.45009937290768498</v>
+      </c>
+      <c r="C89">
+        <v>-7.3464623160084105E-2</v>
+      </c>
+    </row>
+    <row r="90" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A90" t="s">
+        <v>10</v>
+      </c>
+      <c r="B90">
+        <v>-7.3464623160083994E-2</v>
+      </c>
+      <c r="C90">
+        <v>1.24220234669627E-2</v>
+      </c>
+    </row>
+    <row r="92" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A92" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="94" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A94" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A96" t="s">
+        <v>2</v>
+      </c>
+      <c r="B96" t="s">
+        <v>3</v>
+      </c>
+      <c r="C96" t="s">
+        <v>4</v>
+      </c>
+      <c r="D96" t="s">
+        <v>5</v>
+      </c>
+      <c r="E96" t="s">
+        <v>6</v>
+      </c>
+      <c r="F96" t="s">
+        <v>7</v>
+      </c>
+      <c r="G96" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="97" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A97" t="s">
+        <v>9</v>
+      </c>
+      <c r="B97">
+        <v>2.81287966433896</v>
+      </c>
+      <c r="C97">
+        <v>2.10494324397003</v>
+      </c>
+      <c r="D97">
+        <v>3.52081608470789</v>
+      </c>
+      <c r="E97">
+        <v>16.657818142705</v>
+      </c>
+      <c r="F97">
+        <v>8.2066372202297106</v>
+      </c>
+      <c r="G97">
+        <v>33.8120106724623</v>
+      </c>
+    </row>
+    <row r="98" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A98" t="s">
+        <v>10</v>
+      </c>
+      <c r="B98">
+        <v>-3.5648642280722898E-2</v>
+      </c>
+      <c r="C98">
+        <v>-0.150324965068515</v>
+      </c>
+      <c r="D98">
+        <v>7.90276805070695E-2</v>
+      </c>
+      <c r="E98">
+        <v>0.96497928684704404</v>
+      </c>
+      <c r="F98">
+        <v>0.86042832183997398</v>
+      </c>
+      <c r="G98">
+        <v>1.0822342784493</v>
+      </c>
+    </row>
+    <row r="100" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A100" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="101" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A101" t="s">
+        <v>2</v>
+      </c>
+      <c r="B101" t="s">
+        <v>9</v>
+      </c>
+      <c r="C101" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="102" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A102" t="s">
+        <v>9</v>
+      </c>
+      <c r="B102">
+        <v>0.13046449244358099</v>
+      </c>
+      <c r="C102">
+        <v>-2.07385565727519E-2</v>
+      </c>
+    </row>
+    <row r="103" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A103" t="s">
+        <v>10</v>
+      </c>
+      <c r="B103">
+        <v>-2.07385565727519E-2</v>
+      </c>
+      <c r="C103">
+        <v>3.423350248423E-3</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Q11"/>
   <sheetFormatPr defaultColWidth="11.5546875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="28.21875" customWidth="1"/>
+    <col min="1" max="1" width="55.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:17" x14ac:dyDescent="0.3">
@@ -8059,13 +9011,38 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00D9141B-AB39-473B-A049-B1C50259687D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{00D9141B-AB39-473B-A049-B1C50259687D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="a4e98822-f433-4c96-8830-5cb2d7491f7d"/>
+    <ds:schemaRef ds:uri="adc125f1-7df9-46f4-a9a7-022dd426a2bb"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B1892EB-68FF-40B4-8EED-2D5A004731C8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3B1892EB-68FF-40B4-8EED-2D5A004731C8}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B99B4EC1-0E3A-4156-AB7A-75FF64620031}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B99B4EC1-0E3A-4156-AB7A-75FF64620031}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="a4e98822-f433-4c96-8830-5cb2d7491f7d"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>